<commit_message>
Updated word counts for The Sentinel
</commit_message>
<xml_diff>
--- a/code-analysis/word-count-code-comments/Code-comments-word-counts.xlsx
+++ b/code-analysis/word-count-code-comments/Code-comments-word-counts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mark/Documents/Files/Websites/Repositories/bbcelite-scripts/code-analysis/word-count-code-comments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FC01FE-4D66-2045-991A-B77BE1DCB18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2635BFFC-BB55-4345-A01D-CC9435FFDBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17280" yWindow="2800" windowWidth="21580" windowHeight="17800" xr2:uid="{F0A95109-ED5E-2247-9F97-3254041D3CDA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="123">
   <si>
     <t>Lines</t>
   </si>
@@ -402,6 +402,12 @@
   </si>
   <si>
     <t>Commentary plus deep dives:</t>
+  </si>
+  <si>
+    <t>Word counts of popular books:</t>
+  </si>
+  <si>
+    <t>https://brokebybooks.com/the-word-count-of-175-favorite-novels/</t>
   </si>
 </sst>
 </file>
@@ -500,6 +506,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Results"/>
@@ -508,12 +515,10 @@
     <sheetDataSet>
       <sheetData sheetId="0">
         <row r="7">
-          <cell r="B7">
-            <v>428676</v>
-          </cell>
+          <cell r="B7"/>
         </row>
       </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -816,7 +821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4742C6F-ED5A-B74D-BFAE-09A904247301}">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36.6640625" customWidth="1"/>
@@ -848,15 +853,15 @@
       </c>
       <c r="B2" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A2,linecount.txt!E:E,"&lt;&gt;elite-build-options.asm",linecount.txt!E:E,"&lt;&gt;elite-bank-options.asm",linecount.txt!E:E,"&lt;&gt;elite-disc.asm",linecount.txt!E:E,"&lt;&gt;elite-readme.asm")+$G$4</f>
-        <v>151589</v>
+        <v>151594</v>
       </c>
       <c r="C2" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A2)</f>
-        <v>519881</v>
+        <v>519876</v>
       </c>
       <c r="D2" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A2)</f>
-        <v>800265</v>
+        <v>800270</v>
       </c>
       <c r="F2" t="s">
         <v>81</v>
@@ -900,11 +905,11 @@
       </c>
       <c r="C4" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A4)</f>
-        <v>349369</v>
+        <v>349312</v>
       </c>
       <c r="D4" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A4)</f>
-        <v>544543</v>
+        <v>544491</v>
       </c>
       <c r="F4" t="s">
         <v>86</v>
@@ -920,15 +925,15 @@
       </c>
       <c r="B5" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A5,linecount.txt!E:E,"&lt;&gt;revs-build-options.asm",linecount.txt!E:E,"&lt;&gt;revs-disc.asm")</f>
-        <v>67559</v>
+        <v>67591</v>
       </c>
       <c r="C5" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A5)</f>
-        <v>270219</v>
+        <v>270294</v>
       </c>
       <c r="D5" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A5)</f>
-        <v>369255</v>
+        <v>369366</v>
       </c>
       <c r="G5" s="4"/>
     </row>
@@ -938,15 +943,15 @@
       </c>
       <c r="B6" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A6,linecount.txt!E:E,"&lt;&gt;elite-build-options.asm",linecount.txt!E:E,"&lt;&gt;elite-bank-options.asm",linecount.txt!E:E,"&lt;&gt;elite-disc.asm",linecount.txt!E:E,"&lt;&gt;elite-readme.asm")</f>
-        <v>66278</v>
+        <v>66284</v>
       </c>
       <c r="C6" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A6)</f>
-        <v>248188</v>
+        <v>248218</v>
       </c>
       <c r="D6" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A6)</f>
-        <v>355882</v>
+        <v>355918</v>
       </c>
       <c r="F6" t="s">
         <v>82</v>
@@ -986,15 +991,15 @@
       </c>
       <c r="B8" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A8,linecount.txt!E:E,"&lt;&gt;elite-build-options.asm",linecount.txt!E:E,"&lt;&gt;elite-bank-options.asm",linecount.txt!E:E,"&lt;&gt;elite-disc.asm",linecount.txt!E:E,"&lt;&gt;elite-readme.asm")</f>
-        <v>64571</v>
+        <v>64582</v>
       </c>
       <c r="C8" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A8)</f>
-        <v>246415</v>
+        <v>246450</v>
       </c>
       <c r="D8" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A8)</f>
-        <v>355943</v>
+        <v>355994</v>
       </c>
       <c r="F8" t="s">
         <v>86</v>
@@ -1028,15 +1033,15 @@
       </c>
       <c r="B10" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A10,linecount.txt!E:E,"&lt;&gt;elite-build-options.asm",linecount.txt!E:E,"&lt;&gt;elite-bank-options.asm",linecount.txt!E:E,"&lt;&gt;elite-disc.asm",linecount.txt!E:E,"&lt;&gt;elite-readme.asm")</f>
-        <v>59626</v>
+        <v>59632</v>
       </c>
       <c r="C10" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A10)</f>
-        <v>228717</v>
+        <v>228719</v>
       </c>
       <c r="D10" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A10)</f>
-        <v>325884</v>
+        <v>325897</v>
       </c>
       <c r="F10" t="s">
         <v>84</v>
@@ -1045,19 +1050,19 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="B11" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A11,linecount.txt!E:E,"&lt;&gt;elite-build-options.asm",linecount.txt!E:E,"&lt;&gt;elite-bank-options.asm",linecount.txt!E:E,"&lt;&gt;elite-disc.asm",linecount.txt!E:E,"&lt;&gt;elite-readme.asm")</f>
-        <v>41863</v>
+        <v>41902</v>
       </c>
       <c r="C11" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A11)</f>
-        <v>172072</v>
+        <v>182847</v>
       </c>
       <c r="D11" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A11)</f>
-        <v>232952</v>
+        <v>245008</v>
       </c>
       <c r="F11" t="s">
         <v>2</v>
@@ -1069,19 +1074,19 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="B12" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A12,linecount.txt!E:E,"&lt;&gt;elite-build-options.asm",linecount.txt!E:E,"&lt;&gt;elite-bank-options.asm",linecount.txt!E:E,"&lt;&gt;elite-disc.asm",linecount.txt!E:E,"&lt;&gt;elite-readme.asm")</f>
-        <v>41020</v>
+        <v>41869</v>
       </c>
       <c r="C12" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A12)</f>
-        <v>178109</v>
+        <v>172083</v>
       </c>
       <c r="D12" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A12)</f>
-        <v>239380</v>
+        <v>232975</v>
       </c>
       <c r="F12" t="s">
         <v>8</v>
@@ -1097,15 +1102,15 @@
       </c>
       <c r="B13" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A13,linecount.txt!E:E,"&lt;&gt;elite-build-options.asm",linecount.txt!E:E,"&lt;&gt;elite-bank-options.asm",linecount.txt!E:E,"&lt;&gt;elite-disc.asm",linecount.txt!E:E,"&lt;&gt;elite-readme.asm")</f>
-        <v>37476</v>
+        <v>37481</v>
       </c>
       <c r="C13" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A13)</f>
-        <v>151004</v>
+        <v>150999</v>
       </c>
       <c r="D13" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A13)</f>
-        <v>205681</v>
+        <v>205686</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1114,15 +1119,15 @@
       </c>
       <c r="B14" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A14,linecount.txt!E:E,"&lt;&gt;aviator-build-options.asm",linecount.txt!E:E,"&lt;&gt;aviator-disc.asm",linecount.txt!E:E,"&lt;&gt;aviator-readme.asm")</f>
-        <v>31407</v>
+        <v>31405</v>
       </c>
       <c r="C14" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A14)</f>
-        <v>133534</v>
+        <v>133512</v>
       </c>
       <c r="D14" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A14)</f>
-        <v>178304</v>
+        <v>178280</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1131,29 +1136,29 @@
       </c>
       <c r="B15" s="4">
         <f>SUMIFS(linecount.txt!A:A,linecount.txt!D:D,Totals!$A15,linecount.txt!E:E,"&lt;&gt;revs-build-options.asm",linecount.txt!E:E,"&lt;&gt;revs-disc.asm")</f>
-        <v>15270</v>
+        <v>15268</v>
       </c>
       <c r="C15" s="4">
         <f>SUMIFS(wordcount.txt!A:A,wordcount.txt!B:B,Totals!$A15)</f>
-        <v>53052</v>
+        <v>53043</v>
       </c>
       <c r="D15" s="4">
         <f>SUMIFS(linecount.txt!B:B,linecount.txt!D:D,Totals!$A15)</f>
-        <v>83770</v>
+        <v>83759</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B16" s="5">
         <f>SUM(B2:B15)</f>
-        <v>917273</v>
+        <v>918222</v>
       </c>
       <c r="C16" s="5">
         <f>SUM(C2:C15)</f>
-        <v>3413374</v>
+        <v>3418167</v>
       </c>
       <c r="D16" s="5">
         <f>SUM(D2:D15)</f>
-        <v>4984394</v>
+        <v>4990179</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -1272,8 +1277,8 @@
         <v>119</v>
       </c>
       <c r="G35" s="6">
-        <f>C3+C14+C5+C15+C12</f>
-        <v>1035680</v>
+        <f>C3+C14+C5+C15+C11</f>
+        <v>1040462</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1288,12 +1293,22 @@
       </c>
       <c r="G36" s="6">
         <f>C16+[1]Results!$B$7</f>
-        <v>3842050</v>
+        <v>3418167</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1374,7 +1389,7 @@
         <v>213311</v>
       </c>
       <c r="C4" s="2">
-        <v>1480763</v>
+        <v>1480762</v>
       </c>
       <c r="D4" t="s">
         <v>94</v>
@@ -1402,13 +1417,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>3368</v>
+        <v>3374</v>
       </c>
       <c r="B6" s="2">
-        <v>18072</v>
+        <v>18095</v>
       </c>
       <c r="C6" s="2">
-        <v>124951</v>
+        <v>125142</v>
       </c>
       <c r="D6" t="s">
         <v>94</v>
@@ -1476,7 +1491,7 @@
         <v>192980</v>
       </c>
       <c r="C10" s="2">
-        <v>1336773</v>
+        <v>1336772</v>
       </c>
       <c r="D10" t="s">
         <v>95</v>
@@ -1606,13 +1621,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>1520</v>
+        <v>1515</v>
       </c>
       <c r="B18" s="2">
-        <v>6044</v>
+        <v>5987</v>
       </c>
       <c r="C18" s="2">
-        <v>40691</v>
+        <v>40341</v>
       </c>
       <c r="D18" t="s">
         <v>95</v>
@@ -1623,13 +1638,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>2591</v>
+        <v>2596</v>
       </c>
       <c r="B19" s="2">
-        <v>13674</v>
+        <v>13679</v>
       </c>
       <c r="C19" s="2">
-        <v>94075</v>
+        <v>94180</v>
       </c>
       <c r="D19" t="s">
         <v>95</v>
@@ -1680,7 +1695,7 @@
         <v>177824</v>
       </c>
       <c r="C22" s="2">
-        <v>1243784</v>
+        <v>1243783</v>
       </c>
       <c r="D22" t="s">
         <v>95</v>
@@ -1912,13 +1927,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>1336</v>
+        <v>1347</v>
       </c>
       <c r="B36" s="2">
-        <v>6930</v>
+        <v>6981</v>
       </c>
       <c r="C36" s="2">
-        <v>47381</v>
+        <v>47932</v>
       </c>
       <c r="D36" t="s">
         <v>96</v>
@@ -1952,7 +1967,7 @@
         <v>290239</v>
       </c>
       <c r="C38" s="2">
-        <v>2010000</v>
+        <v>2009999</v>
       </c>
       <c r="D38" t="s">
         <v>96</v>
@@ -2088,7 +2103,7 @@
         <v>194457</v>
       </c>
       <c r="C46" s="2">
-        <v>1350782</v>
+        <v>1350781</v>
       </c>
       <c r="D46" t="s">
         <v>97</v>
@@ -2116,13 +2131,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
-        <v>2080</v>
+        <v>2085</v>
       </c>
       <c r="B48" s="2">
-        <v>10297</v>
+        <v>10302</v>
       </c>
       <c r="C48" s="2">
-        <v>70189</v>
+        <v>70294</v>
       </c>
       <c r="D48" t="s">
         <v>97</v>
@@ -2207,7 +2222,7 @@
         <v>284939</v>
       </c>
       <c r="C53" s="2">
-        <v>1995379</v>
+        <v>1995378</v>
       </c>
       <c r="D53" t="s">
         <v>98</v>
@@ -2269,13 +2284,13 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B57" s="2">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="C57" s="2">
-        <v>2791</v>
+        <v>2853</v>
       </c>
       <c r="D57" t="s">
         <v>98</v>
@@ -2286,13 +2301,13 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B58" s="2">
-        <v>656</v>
+        <v>668</v>
       </c>
       <c r="C58" s="2">
-        <v>5036</v>
+        <v>5098</v>
       </c>
       <c r="D58" t="s">
         <v>98</v>
@@ -2303,13 +2318,13 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
-        <v>1536</v>
+        <v>1538</v>
       </c>
       <c r="B59" s="2">
-        <v>4667</v>
+        <v>4679</v>
       </c>
       <c r="C59" s="2">
-        <v>33603</v>
+        <v>33665</v>
       </c>
       <c r="D59" t="s">
         <v>98</v>
@@ -2411,7 +2426,7 @@
         <v>262384</v>
       </c>
       <c r="C65" s="2">
-        <v>1834233</v>
+        <v>1834232</v>
       </c>
       <c r="D65" t="s">
         <v>103</v>
@@ -2541,13 +2556,13 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" s="2">
-        <v>48605</v>
+        <v>48609</v>
       </c>
       <c r="B73" s="2">
-        <v>271938</v>
+        <v>271974</v>
       </c>
       <c r="C73" s="2">
-        <v>1883911</v>
+        <v>1884194</v>
       </c>
       <c r="D73" t="s">
         <v>106</v>
@@ -2575,13 +2590,13 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" s="2">
-        <v>1297</v>
+        <v>1299</v>
       </c>
       <c r="B75" s="2">
-        <v>6942</v>
+        <v>6919</v>
       </c>
       <c r="C75" s="2">
-        <v>47351</v>
+        <v>47248</v>
       </c>
       <c r="D75" t="s">
         <v>106</v>
@@ -2700,7 +2715,7 @@
         <v>212006</v>
       </c>
       <c r="C82" s="2">
-        <v>1480519</v>
+        <v>1480518</v>
       </c>
       <c r="D82" t="s">
         <v>107</v>
@@ -2921,7 +2936,7 @@
         <v>141015</v>
       </c>
       <c r="C95" s="2">
-        <v>1010351</v>
+        <v>1010350</v>
       </c>
       <c r="D95" t="s">
         <v>107</v>
@@ -2938,7 +2953,7 @@
         <v>204966</v>
       </c>
       <c r="C96" s="2">
-        <v>1448803</v>
+        <v>1448802</v>
       </c>
       <c r="D96" t="s">
         <v>107</v>
@@ -3023,7 +3038,7 @@
         <v>315656</v>
       </c>
       <c r="C101" s="2">
-        <v>2222891</v>
+        <v>2222890</v>
       </c>
       <c r="D101" t="s">
         <v>112</v>
@@ -3102,13 +3117,13 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="2">
-        <v>3403</v>
+        <v>3408</v>
       </c>
       <c r="B106" s="2">
-        <v>17693</v>
+        <v>17698</v>
       </c>
       <c r="C106" s="2">
-        <v>125692</v>
+        <v>125797</v>
       </c>
       <c r="D106" t="s">
         <v>107</v>
@@ -3278,7 +3293,7 @@
         <v>143017</v>
       </c>
       <c r="C116" s="2">
-        <v>989387</v>
+        <v>989386</v>
       </c>
       <c r="D116" t="s">
         <v>108</v>
@@ -3374,13 +3389,13 @@
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" s="2">
-        <v>31407</v>
+        <v>31405</v>
       </c>
       <c r="B122" s="2">
-        <v>178126</v>
+        <v>178102</v>
       </c>
       <c r="C122" s="2">
-        <v>1248656</v>
+        <v>1248487</v>
       </c>
       <c r="D122" t="s">
         <v>110</v>
@@ -3391,13 +3406,13 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" s="2">
-        <v>43728</v>
+        <v>43760</v>
       </c>
       <c r="B123" s="2">
-        <v>227075</v>
+        <v>227186</v>
       </c>
       <c r="C123" s="2">
-        <v>1677469</v>
+        <v>1678559</v>
       </c>
       <c r="D123" t="s">
         <v>109</v>
@@ -3578,13 +3593,13 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" s="2">
-        <v>40975</v>
+        <v>41857</v>
       </c>
       <c r="B134" s="2">
-        <v>239203</v>
+        <v>244831</v>
       </c>
       <c r="C134" s="2">
-        <v>1771063</v>
+        <v>1810916</v>
       </c>
       <c r="D134" t="s">
         <v>115</v>
@@ -3612,13 +3627,13 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" s="2">
-        <v>15087</v>
+        <v>15085</v>
       </c>
       <c r="B136" s="2">
-        <v>83112</v>
+        <v>83101</v>
       </c>
       <c r="C136" s="2">
-        <v>721387</v>
+        <v>721259</v>
       </c>
       <c r="D136" t="s">
         <v>111</v>
@@ -3719,7 +3734,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>13523</v>
+        <v>13534</v>
       </c>
       <c r="B6" t="s">
         <v>94</v>
@@ -3851,7 +3866,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>3327</v>
+        <v>3275</v>
       </c>
       <c r="B18" t="s">
         <v>95</v>
@@ -3862,7 +3877,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>9711</v>
+        <v>9706</v>
       </c>
       <c r="B19" t="s">
         <v>95</v>
@@ -4049,7 +4064,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>5063</v>
+        <v>5098</v>
       </c>
       <c r="B36" t="s">
         <v>96</v>
@@ -4181,7 +4196,7 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
-        <v>7451</v>
+        <v>7446</v>
       </c>
       <c r="B48" t="s">
         <v>97</v>
@@ -4280,7 +4295,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="B57" t="s">
         <v>98</v>
@@ -4291,7 +4306,7 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="B58" t="s">
         <v>98</v>
@@ -4302,7 +4317,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
-        <v>2605</v>
+        <v>2615</v>
       </c>
       <c r="B59" t="s">
         <v>98</v>
@@ -4456,7 +4471,7 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="2">
-        <v>207135</v>
+        <v>207167</v>
       </c>
       <c r="B73" t="s">
         <v>106</v>
@@ -4478,7 +4493,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="2">
-        <v>5174</v>
+        <v>5144</v>
       </c>
       <c r="B75" t="s">
         <v>106</v>
@@ -4819,7 +4834,7 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="2">
-        <v>13321</v>
+        <v>13316</v>
       </c>
       <c r="B106" t="s">
         <v>107</v>
@@ -4995,7 +5010,7 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" s="2">
-        <v>133425</v>
+        <v>133403</v>
       </c>
       <c r="B122" t="s">
         <v>110</v>
@@ -5006,7 +5021,7 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" s="2">
-        <v>170214</v>
+        <v>170289</v>
       </c>
       <c r="B123" t="s">
         <v>109</v>
@@ -5127,7 +5142,7 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" s="2">
-        <v>177994</v>
+        <v>182732</v>
       </c>
       <c r="B134" t="s">
         <v>115</v>
@@ -5149,7 +5164,7 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" s="2">
-        <v>52623</v>
+        <v>52614</v>
       </c>
       <c r="B136" t="s">
         <v>111</v>

</xml_diff>